<commit_message>
Ajustando exportacion de inspecciones
</commit_message>
<xml_diff>
--- a/public/plantillas/22_INSPECCION_SEMANAL.xlsx
+++ b/public/plantillas/22_INSPECCION_SEMANAL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{660C8B18-896E-4740-9C40-E8D7A968B92A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{496EC8C8-266B-944B-95BB-97E4D77551BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEHÍCULOS" sheetId="1" r:id="rId1"/>
@@ -37,9 +37,6 @@
     <t>FECHA:</t>
   </si>
   <si>
-    <t>FRENTE:</t>
-  </si>
-  <si>
     <t>CONTRATISTA: RECAL ESTRUCTURAS</t>
   </si>
   <si>
@@ -146,6 +143,9 @@
   </si>
   <si>
     <t>SI</t>
+  </si>
+  <si>
+    <t>FRENTE: TRAMO 1,2 Y 3</t>
   </si>
 </sst>
 </file>
@@ -331,22 +331,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -354,8 +348,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -662,7 +662,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3"/>
@@ -674,7 +674,7 @@
       <c r="H1" s="4"/>
     </row>
     <row r="2" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3"/>
@@ -686,13 +686,13 @@
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
-        <v>36</v>
+      <c r="A3" s="13" t="s">
+        <v>35</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="4"/>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="13" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="3"/>
@@ -700,22 +700,22 @@
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
-        <v>3</v>
+      <c r="A4" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="4"/>
-      <c r="E4" s="6" t="s">
-        <v>4</v>
+      <c r="E4" s="13" t="s">
+        <v>3</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
-        <v>5</v>
+      <c r="A5" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -726,144 +726,144 @@
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
-        <v>6</v>
+      <c r="A6" s="5" t="s">
+        <v>5</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="4"/>
       <c r="D6" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>7</v>
+        <v>38</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
       <c r="H6" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
-        <v>8</v>
+      <c r="A7" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>9</v>
+        <v>38</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>8</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
       <c r="H7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="8" t="s">
-        <v>10</v>
+      <c r="A8" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>11</v>
+        <v>38</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="4"/>
       <c r="H8" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
-        <v>12</v>
+      <c r="A9" s="5" t="s">
+        <v>11</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="4"/>
       <c r="D9" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>13</v>
+        <v>38</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="4"/>
       <c r="H9" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="8" t="s">
-        <v>14</v>
+      <c r="A10" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="4"/>
       <c r="D10" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>15</v>
+        <v>38</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>14</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="4"/>
       <c r="H10" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
-        <v>16</v>
+      <c r="A11" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="4"/>
       <c r="D11" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>17</v>
+        <v>38</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="4"/>
       <c r="H11" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="8"/>
+      <c r="C12" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="9" t="s">
+      <c r="D12" s="8"/>
+      <c r="E12" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="9" t="s">
+      <c r="F12" s="8"/>
+      <c r="G12" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" s="10"/>
+      <c r="H12" s="8"/>
     </row>
     <row r="13" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="12"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="10"/>
     </row>
     <row r="14" spans="1:8" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13" t="s">
-        <v>22</v>
+      <c r="A14" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -1861,14 +1861,12 @@
     <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:H4"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A10:C10"/>
@@ -1879,12 +1877,14 @@
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="E12:F13"/>
     <mergeCell ref="G12:H13"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="E9:G9"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -1907,7 +1907,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3"/>
@@ -1919,8 +1919,8 @@
       <c r="H1" s="4"/>
     </row>
     <row r="2" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
-        <v>38</v>
+      <c r="A2" s="12" t="s">
+        <v>37</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -1931,13 +1931,13 @@
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
-        <v>36</v>
+      <c r="A3" s="13" t="s">
+        <v>35</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="4"/>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="13" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="3"/>
@@ -1945,22 +1945,22 @@
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
-        <v>3</v>
+      <c r="A4" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="4"/>
-      <c r="E4" s="6" t="s">
-        <v>37</v>
+      <c r="E4" s="13" t="s">
+        <v>36</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
-        <v>5</v>
+      <c r="A5" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -1971,144 +1971,144 @@
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
-        <v>23</v>
+      <c r="A6" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="4"/>
       <c r="D6" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>24</v>
+        <v>38</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>23</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
       <c r="H6" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
-        <v>25</v>
+      <c r="A7" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>26</v>
+        <v>38</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
       <c r="H7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="8" t="s">
-        <v>27</v>
+      <c r="A8" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>28</v>
+        <v>38</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>27</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="4"/>
       <c r="H8" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
-        <v>29</v>
+      <c r="A9" s="5" t="s">
+        <v>28</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="4"/>
       <c r="D9" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>30</v>
+        <v>38</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="4"/>
       <c r="H9" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="8" t="s">
-        <v>31</v>
+      <c r="A10" s="5" t="s">
+        <v>30</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="4"/>
       <c r="D10" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>32</v>
+        <v>38</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="4"/>
       <c r="H10" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
-        <v>33</v>
+      <c r="A11" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="4"/>
       <c r="D11" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>34</v>
+        <v>38</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>33</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="4"/>
       <c r="H11" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="8"/>
+      <c r="C12" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" s="10"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H12" s="8"/>
     </row>
     <row r="13" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="12"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="10"/>
     </row>
     <row r="14" spans="1:8" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13" t="s">
-        <v>22</v>
+      <c r="A14" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -3106,14 +3106,12 @@
     <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:H4"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A10:C10"/>
@@ -3124,12 +3122,14 @@
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="E12:F13"/>
     <mergeCell ref="G12:H13"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="E9:G9"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>